<commit_message>
Also add the renamed data sets to the design
</commit_message>
<xml_diff>
--- a/Design2.xlsx
+++ b/Design2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\Org\EXP\EN-DS\Datensicherung\Martin Gühmann\SyntheticDataMouseKidneyGlomeruli\YoloGlomeruliAuswertung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50DA632-5501-40CF-82AB-162A484DF483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB13EA7A-A2AB-4F53-A9B8-42D868B1037C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="68">
   <si>
     <t>Versuch</t>
   </si>
@@ -62,12 +62,6 @@
     <t>800_SG_au</t>
   </si>
   <si>
-    <t>B10_Val</t>
-  </si>
-  <si>
-    <t>B007_Test</t>
-  </si>
-  <si>
     <t>train-001.txt</t>
   </si>
   <si>
@@ -212,10 +206,34 @@
     <t>m</t>
   </si>
   <si>
-    <t>OG_aug</t>
-  </si>
-  <si>
-    <t>SG_aug</t>
+    <t>Val</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>SynAug</t>
+  </si>
+  <si>
+    <t>Syn</t>
+  </si>
+  <si>
+    <t>TinyAug</t>
+  </si>
+  <si>
+    <t>TrainTiny</t>
+  </si>
+  <si>
+    <t>TrainSmall</t>
+  </si>
+  <si>
+    <t>GloAug</t>
+  </si>
+  <si>
+    <t>Glo</t>
+  </si>
+  <si>
+    <t>TrainBig</t>
   </si>
 </sst>
 </file>
@@ -616,34 +634,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -651,7 +669,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
@@ -689,7 +707,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -727,7 +745,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -765,7 +783,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -803,7 +821,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -841,7 +859,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
@@ -879,7 +897,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
@@ -917,7 +935,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -955,7 +973,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
@@ -993,7 +1011,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
@@ -1031,7 +1049,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
@@ -1069,7 +1087,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1107,7 +1125,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1145,7 +1163,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1183,7 +1201,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1221,7 +1239,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1259,7 +1277,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1297,7 +1315,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1335,7 +1353,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1434,37 +1452,37 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1472,37 +1490,37 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1510,37 +1528,37 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1548,37 +1566,37 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1586,37 +1604,37 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1624,37 +1642,37 @@
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1662,37 +1680,37 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1700,37 +1718,37 @@
         <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:1024" x14ac:dyDescent="0.2">
@@ -1763,7 +1781,7 @@
     </row>
     <row r="14" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F14" s="3">
         <v>0</v>
@@ -1785,7 +1803,7 @@
     </row>
     <row r="15" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1805,7 +1823,7 @@
     </row>
     <row r="25" spans="4:20" x14ac:dyDescent="0.2">
       <c r="J25" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="4:20" x14ac:dyDescent="0.2">
@@ -1814,49 +1832,49 @@
         <v>1</v>
       </c>
       <c r="F31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H31" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="I31" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="J31" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="K31" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="L31" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="M31" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="N31" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="O31" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="N31" s="4" t="s">
+      <c r="P31" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="Q31" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="P31" s="4" t="s">
+      <c r="R31" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Q31" s="4" t="s">
+      <c r="S31" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="R31" s="4" t="s">
+      <c r="T31" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="S31" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="T31" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="32" spans="4:20" x14ac:dyDescent="0.2">
@@ -1910,85 +1928,85 @@
     </row>
     <row r="33" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D33" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E33" s="4">
         <v>15</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
       <c r="M33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N33" s="4"/>
       <c r="O33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q33" s="4"/>
       <c r="R33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="T33" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D34" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E34" s="4">
         <v>60</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
       <c r="J34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="O34" s="4"/>
       <c r="P34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R34" s="4"/>
       <c r="S34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="T34" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D35" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E35" s="4">
         <v>800</v>
@@ -1996,38 +2014,38 @@
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="S35" s="4"/>
       <c r="T35" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D36" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E36" s="4">
         <v>3200</v>
@@ -2036,32 +2054,32 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M36" s="4"/>
       <c r="N36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="P36" s="4"/>
       <c r="Q36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="T36" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2081,16 +2099,16 @@
   <sheetData>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" s="4">
         <v>0</v>
@@ -2099,7 +2117,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B6" s="4">
         <v>1</v>
@@ -2108,7 +2126,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B7" s="4">
         <v>0</v>
@@ -2117,7 +2135,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B8" s="4">
         <v>1</v>
@@ -2126,7 +2144,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B9" s="4">
         <v>2</v>
@@ -2135,7 +2153,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B10" s="4">
         <v>2</v>

</xml_diff>